<commit_message>
docs: make engineering artifacts Markdown-first with audience Excel views
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
@@ -21,10 +21,11 @@
     <sheet name="11 Risks and Limits" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="12 Pilot and Rollout" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="13 Gate Mapping" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="14 Audience Profiles" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm.Print_Titles" localSheetId="0">'00 Read Me'!$1:$4,'00 Read Me'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">'00 Read Me'!$A$1:$C$20</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">'00 Read Me'!$A$1:$C$23</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="1">'01 Sources'!$1:$4,'01 Sources'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="1">'01 Sources'!$A$1:$H$47</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="2">'02 Findings'!$1:$4,'02 Findings'!$A:$A</definedName>
@@ -40,17 +41,19 @@
     <definedName name="_xlnm.Print_Titles" localSheetId="7">'07 Update Requirements'!$1:$4,'07 Update Requirements'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="7">'07 Update Requirements'!$A$1:$G$24</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="8">'08 Verification Plan'!$1:$4,'08 Verification Plan'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="8">'08 Verification Plan'!$A$1:$E$31</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="8">'08 Verification Plan'!$A$1:$E$33</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="9">'09 Delivery Plan'!$1:$4,'09 Delivery Plan'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="9">'09 Delivery Plan'!$A$1:$G$10</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="10">'10 Decisions'!$1:$4,'10 Decisions'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="10">'10 Decisions'!$A$1:$F$12</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="11">'11 Risks and Limits'!$1:$4,'11 Risks and Limits'!$A:$A</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="11">'11 Risks and Limits'!$A$1:$E$16</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="11">'11 Risks and Limits'!$A$1:$E$17</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="12">'12 Pilot and Rollout'!$1:$4,'12 Pilot and Rollout'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="12">'12 Pilot and Rollout'!$A$1:$E$9</definedName>
     <definedName name="_xlnm.Print_Titles" localSheetId="13">'13 Gate Mapping'!$1:$4,'13 Gate Mapping'!$A:$A</definedName>
     <definedName name="_xlnm.Print_Area" localSheetId="13">'13 Gate Mapping'!$A$1:$E$11</definedName>
+    <definedName name="_xlnm.Print_Titles" localSheetId="14">'14 Audience Profiles'!$1:$4,'14 Audience Profiles'!$A:$A</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="14">'14 Audience Profiles'!$A$1:$E$9</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -229,8 +232,8 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EngineeringResearch00" displayName="EngineeringResearch00" ref="A4:C20" headerRowCount="1">
-  <autoFilter ref="A4:C20"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="1" name="EngineeringResearch00" displayName="EngineeringResearch00" ref="A4:C23" headerRowCount="1">
+  <autoFilter ref="A4:C23"/>
   <tableColumns count="3">
     <tableColumn id="1" name="Item"/>
     <tableColumn id="2" name="Value"/>
@@ -272,8 +275,8 @@
 </file>
 
 <file path=xl/tables/table12.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="EngineeringResearch11" displayName="EngineeringResearch11" ref="A4:E16" headerRowCount="1">
-  <autoFilter ref="A4:E16"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="12" name="EngineeringResearch11" displayName="EngineeringResearch11" ref="A4:E17" headerRowCount="1">
+  <autoFilter ref="A4:E17"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Risk ID"/>
     <tableColumn id="2" name="Risk"/>
@@ -308,6 +311,20 @@
     <tableColumn id="3" name="Artifact content to inspect"/>
     <tableColumn id="4" name="Existing harness integration"/>
     <tableColumn id="5" name="Review boundary"/>
+  </tableColumns>
+  <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table15.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="15" name="EngineeringResearch14" displayName="EngineeringResearch14" ref="A4:E9" headerRowCount="1">
+  <autoFilter ref="A4:E9"/>
+  <tableColumns count="5">
+    <tableColumn id="1" name="Audience ID"/>
+    <tableColumn id="2" name="Audience"/>
+    <tableColumn id="3" name="Selected content"/>
+    <tableColumn id="4" name="Always retain when relevant"/>
+    <tableColumn id="5" name="Source and review boundary"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
 </table>
@@ -422,8 +439,8 @@
 </file>
 
 <file path=xl/tables/table9.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EngineeringResearch08" displayName="EngineeringResearch08" ref="A4:E31" headerRowCount="1">
-  <autoFilter ref="A4:E31"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="9" name="EngineeringResearch08" displayName="EngineeringResearch08" ref="A4:E33" headerRowCount="1">
+  <autoFilter ref="A4:E33"/>
   <tableColumns count="5">
     <tableColumn id="1" name="Verification ID"/>
     <tableColumn id="2" name="Scenario"/>
@@ -724,7 +741,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:C20"/>
+  <dimension ref="A1:C23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="27" customWidth="1" min="1" max="1"/>
@@ -810,7 +827,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.1 / Draft for review</t>
+          <t>0.2 / Draft for review</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -861,12 +878,12 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Excel is the current human review format</t>
+          <t>Markdown is the primary authoring and version-controlled format</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>JSON is a lossless review snapshot for this package; not a second editable authority.</t>
+          <t>RESEARCH.md and PLAN.md are canonical for this package. XLSX and JSON are derived sharing/rendering outputs.</t>
         </is>
       </c>
     </row>
@@ -989,7 +1006,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="39" customHeight="1">
+    <row r="17" ht="54" customHeight="1">
       <c r="A17" s="6" t="inlineStr">
         <is>
           <t>Preserve edits</t>
@@ -997,12 +1014,12 @@
       </c>
       <c r="B17" s="6" t="inlineStr">
         <is>
-          <t>Do not regenerate over an annotated workbook</t>
+          <t>Workbook review is proposed feedback, not another master</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>First reconcile review edits into the JSON snapshot; renderer refuses overwrite.</t>
+          <t>Archive the annotated workbook, compare by stable ID, review proposed changes into Markdown and regenerate a new export. Never silently import agreement or overwrite comments.</t>
         </is>
       </c>
     </row>
@@ -1054,6 +1071,57 @@
       <c r="C20" s="6" t="inlineStr">
         <is>
           <t>LibreOffice rendering and structural checks are evidence, not Excel certification.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="54" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>Audience</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>Research-review: complete evidence and proposed catalogue update</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>Other audience profiles are defined in 14 Audience Profiles for later implementation; this helper renders this review package only.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="39" customHeight="1">
+      <c r="A22" s="6" t="inlineStr">
+        <is>
+          <t>Canonical sources</t>
+        </is>
+      </c>
+      <c r="B22" s="6" t="inlineStr">
+        <is>
+          <t>RESEARCH.md (rationale) and PLAN.md (all detailed records)</t>
+        </is>
+      </c>
+      <c r="C22" s="6" t="inlineStr">
+        <is>
+          <t>Edit Markdown first. The renderer derives the JSON snapshot and workbook directly from PLAN.md.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="54" customHeight="1">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>Export provenance</t>
+        </is>
+      </c>
+      <c r="B23" s="6" t="inlineStr">
+        <is>
+          <t>Source path/hash, audience and generated UTC time are in workbook document properties and JSON metadata</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Compare the source SHA-256 with the current PLAN.md bytes to detect staleness. Do not treat an export as current without checking its source.</t>
         </is>
       </c>
     </row>
@@ -1168,7 +1236,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="69" customHeight="1">
+    <row r="5" ht="114" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>P01</t>
@@ -1176,7 +1244,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>Agree content/schema and existing-engine adapter</t>
+          <t>Agree Markdown content contract, source authority and export adapter</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -1191,21 +1259,21 @@
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>Map existing PRD/story statuses and IDs to Excel rows; define common metadata, typed relations, profiles and narrative sections. Record any consequential adapter decision before code.</t>
+          <t>Map existing PRD/story identities and machine-field authority to canonical Markdown records; define stable criterion IDs, source sections, typed relations and review history. Specify audience selection, export manifest/freshness and feedback reconciliation. Keep machine schemas/diagrams authoritative for their own content. Record consequential adapter decisions before code.</t>
         </is>
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Reviewed contract, source-to-field mapping and tiny/feature/design/release examples.</t>
+          <t>Reviewed Markdown contract and complete tiny/feature/design/release examples; five audience mappings, source-to-field mapping and conflict/freshness rules.</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
         <is>
-          <t>REQ02; REQ03; REQ04; REQ13; REQ14; REQ20</t>
-        </is>
-      </c>
-    </row>
-    <row r="6" ht="69" customHeight="1">
+          <t>REQ02; REQ03; REQ04; REQ09; REQ10; REQ13; REQ14; REQ20</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="114" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
           <t>P02</t>
@@ -1213,7 +1281,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Deterministic Excel workflow with preservation checks</t>
+          <t>Markdown-to-Excel export and feedback reporting</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1228,12 +1296,12 @@
       </c>
       <c r="E6" s="6" t="inlineStr">
         <is>
-          <t>Implement narrow read/write/validate/snapshot helpers; verify schema/version before edit; block stale overwrite; preserve unknown sheets and reviewer cells; no automatic remote actions. Explicitly scope unsupported workbook features.</t>
+          <t>Implement narrow Markdown read/validate, audience export and feedback-diff helpers. Validate source version/hash and stable IDs; flag stale/conflicting feedback; preserve annotated outputs and unsupported workbook content. Source changes require explicit review; no automatic approval import, remote actions or two-way master synchronization. Scope supported features and optional dependency.</t>
         </is>
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Functional tests with temp workbooks: duplicate IDs, broken references, missing evidence, leading literal text, reviewer edits, stale source and round trips.</t>
+          <t>Functional fixtures prove source/export parity, audience omissions and blocker visibility, traceability, literal text, freshness, conflicting feedback, no-overwrite and office round trips.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">
@@ -1242,7 +1310,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="69" customHeight="1">
+    <row r="7" ht="84" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
           <t>P03</t>
@@ -1265,7 +1333,7 @@
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>Write valid Karakana metadata and conditional content guides; link shared schema/tool; add synthetic complete examples and evals for inquiry/research/plan/draft boundaries. Start experimental.</t>
+          <t>Write valid Karakana metadata and conditional content guides for Markdown-first authoring, with optional audience workbooks; link shared contract/tool. Add original complete synthetic examples and evals for inquiry/research/plan/draft boundaries. Start experimental.</t>
         </is>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -1316,7 +1384,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="69" customHeight="1">
+    <row r="9" ht="84" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>P05</t>
@@ -1339,12 +1407,12 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Run original synthetic requirement/story, design/ADR and roadmap/release packs. Validate and render Excel; test human comment reconciliation. A LIMS first-release pack is a later expressly requested application, not the synthetic pilot.</t>
+          <t>Author complete synthetic requirements/stories, ADR/design and roadmap/release records in Markdown. Export by audience; validate/render Excel; test source freshness and reviewed feedback reconciliation. A LIMS release pack remains a later requested application.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Record actual results, review gaps, compatibility and accessibility limitations; agree baseline/profile.</t>
+          <t>Source-to-export parity, useful audience views, preserved blockers/limitations, actual office/feedback results and accessibility limits recorded; agree profile baseline.</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">
@@ -1540,7 +1608,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Four focused authoring workflows plus one Excel-format workflow</t>
+          <t>Four focused Markdown authoring workflows plus one audience Excel export/review workflow</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -1567,17 +1635,17 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>What is the current review authority?</t>
+          <t>What is canonical, and what is shared?</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Excel workbook per scoped baseline with source IDs, review metadata and archived snapshots</t>
+          <t>Markdown is primary and version-controlled. Audience Excel workbooks are derived sharing/review views; JSON snapshots are generated intermediates.</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>JSON/text snapshot enables diffs; not independently editable. Existing machine schemas/ADRs may remain authoritative linked sources.</t>
+          <t>Preserve authoritative machine schemas/diagrams with explicit source links. Workbook-first or two freely editable masters would undermine source review/history.</t>
         </is>
       </c>
       <c r="E7" s="7" t="inlineStr">
@@ -1587,7 +1655,7 @@
       </c>
       <c r="F7" s="7" t="inlineStr">
         <is>
-          <t>Never create two freely editable masters; reconcile imported review changes explicitly.</t>
+          <t>Archive feedback, reconcile reviewed proposals into Markdown, regenerate a new source-versioned export; no automatic approval transfer.</t>
         </is>
       </c>
     </row>
@@ -1700,12 +1768,12 @@
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>P01 schema/adapters with complete synthetic examples, followed by P02 workbook integrity tooling</t>
+          <t>P01 Markdown content/source/export contract and examples, then P02 export integrity/feedback helpers</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Skills-only guidance is faster but cannot reliably preserve/validate human Excel edits.</t>
+          <t>Authoring guidance alone cannot prove source freshness, audience projection or preservation of review feedback.</t>
         </is>
       </c>
       <c r="E11" s="7" t="inlineStr">
@@ -1782,7 +1850,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E16"/>
+  <dimension ref="A1:E17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
@@ -1873,7 +1941,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Conflict checks, stable-ID reconciliation, immutable review snapshots and refuse overwrite by default.</t>
+          <t>Archive exports; stable-ID/version feedback reports; reviewed source changes; refuse overwrite and flag conflicts.</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -1981,7 +2049,7 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Lossless text snapshot, cell/ID change report and readable rendered samples.</t>
+          <t>Review canonical Markdown diffs; generate derived JSON/cell change reports and readable audience samples.</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
@@ -2176,6 +2244,33 @@
       <c r="E16" s="6" t="inlineStr">
         <is>
           <t>Document reviewer</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="54" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>RK13</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Stale or misleading audience workbook</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>Divergent facts or omitted release blocker used in decisions</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>Source revision/hash manifest; flag staleness; explicit omissions/full-source links; retain relevant blockers and limitations in every applicable view.</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>Document owner/export maintainer</t>
         </is>
       </c>
     </row>
@@ -2291,7 +2386,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Control; Sources; Requirements; Stories; Acceptance; Links; Evidence; Review</t>
+          <t>Canonical Markdown feature records plus product/engineering/QA sharing views</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -2318,12 +2413,12 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Design/ADR profile with relevant quality/runtime views</t>
+          <t>Canonical Markdown ADR/design with relevant views plus engineering decision summaries</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Plausible alternatives, narrative rationale, history and schema/diagram links.</t>
+          <t>Complete alternatives/rationale/history in Markdown; summaries resolve to the same source revision and schema/diagram links.</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -2345,12 +2440,12 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Planning/release profile plus requirements/test links</t>
+          <t>Canonical Markdown roadmap/release pack plus executive/product/operations exports</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Forecasts, agreed scope, release notes and operations gates clearly separated.</t>
+          <t>Forecasts, commitments, actual release facts and operations blockers remain distinct and visible in applicable views.</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -2359,7 +2454,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="39" customHeight="1">
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>PL04</t>
@@ -2372,12 +2467,12 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Reviewer decision/comments and change snapshot</t>
+          <t>Archived annotated export, feedback report and reviewed Markdown diff</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>Preserve edits and report changes by stable IDs after office round trip.</t>
+          <t>Preserve edits by stable source ID/version; report stale/conflicting feedback after office round trip; regenerate from the reviewed source.</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
@@ -2461,7 +2556,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="60" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -2469,7 +2564,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Existing process remains authoritative; workbook content complements current file-presence checks.</t>
+          <t>Existing process reviews canonical Markdown and scoped source evidence; audience workbooks accompany it. File presence alone remains insufficient.</t>
         </is>
       </c>
     </row>
@@ -2512,7 +2607,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="32" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>G01</t>
@@ -2525,7 +2620,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Control, project/revision, requested action, source authority</t>
+          <t>Canonical Markdown identity/revision, requested action and linked machine-source authority; export profile/freshness when shared</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -2620,7 +2715,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="32" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>G05</t>
@@ -2633,7 +2728,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Test runs, real evidence, diff, reviews and limitations</t>
+          <t>Canonical Markdown diff, actual test/review evidence and limitations; source-to-export parity/freshness and feedback report when shared</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -2698,6 +2793,240 @@
       <c r="E11" s="6" t="inlineStr">
         <is>
           <t>Record true state and project boundaries; no hidden implementation.</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <hyperlinks>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="B3" r:id="rId1"/>
+  </hyperlinks>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageSetup orientation="landscape" paperSize="8" fitToHeight="0" fitToWidth="1"/>
+  <headerFooter>
+    <oddHeader/>
+    <oddFooter>&amp;C&amp;9 Draft research and proposed update | Page &amp;P of &amp;N</oddFooter>
+    <evenHeader/>
+    <evenFooter/>
+    <firstHeader/>
+    <firstFooter/>
+  </headerFooter>
+  <tableParts count="1">
+    <tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId2"/>
+  </tableParts>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr fitToPage="1"/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="28" customWidth="1" min="2" max="2"/>
+    <col width="65" customWidth="1" min="3" max="3"/>
+    <col width="65" customWidth="1" min="4" max="4"/>
+    <col width="65" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="58" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>14 Audience Profiles</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>Draft for review</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="105" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Purpose</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>Proposed sharing profiles for engineering artifacts; this package itself is the full research-review audience export. Implementation will validate audience selection.</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="21" customHeight="1">
+      <c r="A3" s="3" t="inlineStr">
+        <is>
+          <t>Navigation</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="inlineStr">
+        <is>
+          <t>Return to Read Me</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="34" customHeight="1">
+      <c r="A4" s="5" t="inlineStr">
+        <is>
+          <t>Audience ID</t>
+        </is>
+      </c>
+      <c r="B4" s="5" t="inlineStr">
+        <is>
+          <t>Audience</t>
+        </is>
+      </c>
+      <c r="C4" s="5" t="inlineStr">
+        <is>
+          <t>Selected content</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>Always retain when relevant</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>Source and review boundary</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="39" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>AU01</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>Business / product</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Needs; scope; stories; observable acceptance; outcome roadmap; user-facing release changes</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Dependencies; unconfirmed priorities/forecasts; acceptance gaps; delivered versus planned scope</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>Link full source records and revisions; workbook feedback remains proposed input.</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="39" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>AU02</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>Requirements/acceptance; ADR summaries; design/contract links; implementation tasks; technical release changes</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>Decision status; unresolved constraints; security/quality risks; test and compatibility gaps</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>Complete ADR/design narrative and machine schemas stay at their authoritative source paths.</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="39" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>AU03</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>QA / UAT</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Acceptance; test cases/runs; candidate revision/environment; evidence; defects; acceptance decisions</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Not run/blocked/skipped/fail; unresolved criteria; reviewer identity and evidence limits</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>Case definitions and actual results remain separate; feedback is not imported sign-off.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="39" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>AU04</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>Operations / release</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>Candidate/target; readiness; rollout/recovery; migration; monitoring; support/runbook links</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>Release blockers; backup/restore gaps; known limits; authorization and environment status</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
+        <is>
+          <t>No deployment or operational approval follows from export generation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="39" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>AU05</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>Executive / sponsor</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Outcomes; milestones; confidence; key scope/release status; risks; decisions needed</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Material blockers; uncertainty; forecast versus commitment; deployed/accepted distinctions</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>Declare omitted detail and link the complete baseline; summaries cannot conceal blockers.</t>
         </is>
       </c>
     </row>
@@ -3439,7 +3768,7 @@
       </c>
       <c r="G19" s="6" t="inlineStr">
         <is>
-          <t>Adapt content to Excel; the original proposes repository text files.</t>
+          <t>Author ADRs as repository Markdown; workbook summaries link the complete record.</t>
         </is>
       </c>
       <c r="H19" s="4" t="inlineStr">
@@ -4970,7 +5299,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Four authoring skills and a format-specific Excel skill.</t>
+          <t>Four Markdown authoring skills and an audience-specific Excel export/review skill.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -5006,7 +5335,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="39" customHeight="1">
+    <row r="14" ht="54" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>F10</t>
@@ -5014,7 +5343,7 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Evidence should survive human editing</t>
+          <t>Markdown authority and review evidence must survive audience sharing</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -5024,12 +5353,12 @@
       </c>
       <c r="D14" s="6" t="inlineStr">
         <is>
-          <t>Workbook remains review authority; reconciled text snapshot enables version-control review.</t>
+          <t>Versioned Markdown records are canonical; workbook comments produce reviewed change proposals against source IDs and revisions.</t>
         </is>
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>Never overwrite reviewer cells; compare stable IDs and record change provenance.</t>
+          <t>Preserve annotated exports; flag stale source versions and conflicting feedback. No automatic Markdown writes or approval import.</t>
         </is>
       </c>
     </row>
@@ -5474,7 +5803,7 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Reconcile human comments/decisions by stable IDs; protect against stale overwrites.</t>
+          <t>Archive annotated exports; compare feedback by source ID/revision; review changes into Markdown before regeneration.</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
@@ -5908,7 +6237,7 @@
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Use authoritative machine-readable schema; workbook describes and links it.</t>
+          <t>Use authoritative machine-readable schema; Markdown describes and links it, with optional workbook summaries.</t>
         </is>
       </c>
       <c r="G12" s="6" t="inlineStr">
@@ -6398,7 +6727,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="39" customHeight="1">
+    <row r="5" ht="54" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>SK01</t>
@@ -6411,7 +6740,7 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Evidence-backed requirements, stories, acceptance and traceability authoring/revision</t>
+          <t>Evidence-backed requirements, stories, acceptance and traceability authoring/revision in Markdown, with stable source IDs and revision history</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
@@ -6448,7 +6777,7 @@
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>ADR and architecture/design description authoring/review</t>
+          <t>ADR and architecture/design description authoring/review in Markdown, with stable source IDs and revision history</t>
         </is>
       </c>
       <c r="D6" s="6" t="inlineStr">
@@ -6485,7 +6814,7 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Roadmap, milestone and bounded implementation plan</t>
+          <t>Roadmap, milestone and bounded implementation plan in Markdown, with stable source IDs and revision history</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
@@ -6522,7 +6851,7 @@
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Release plan/assurance, notes and adoption/handover pack</t>
+          <t>Release plan/assurance, notes and adoption/handover pack in Markdown, with stable source IDs and revision history</t>
         </is>
       </c>
       <c r="D8" s="6" t="inlineStr">
@@ -6546,7 +6875,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="39" customHeight="1">
+    <row r="9" ht="54" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>SK05</t>
@@ -6559,7 +6888,7 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Excel creation/editing, validation, review snapshots and artifact locators</t>
+          <t>Derived audience Excel exports, integrity/freshness checks and feedback comparison against Markdown</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
@@ -6569,7 +6898,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>references/workbook-contract.md; assets/profile templates; tool adapter; evals</t>
+          <t>references/workbook-contract.md; audience-profiles.md; assets/export templates; tool adapter; evals</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">
@@ -6579,7 +6908,7 @@
       </c>
       <c r="G9" s="7" t="inlineStr">
         <is>
-          <t>Formatting/transport only; domain semantics come from the selected authoring skill.</t>
+          <t>Sharing/review only. Source content stays in Markdown; existing machine schemas and diagrams retain their explicitly linked authority.</t>
         </is>
       </c>
     </row>
@@ -6637,7 +6966,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="45" customHeight="1">
+    <row r="2" ht="90" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -6645,7 +6974,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Proposed project-workbook schema, not a demand to create all tabs for each task.</t>
+          <t>Derived export table contracts selected per audience; canonical narrative and records remain in Markdown. Not every table belongs in every export.</t>
         </is>
       </c>
     </row>
@@ -6693,7 +7022,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="39" customHeight="1">
+    <row r="5" ht="69" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
           <t>WB01</t>
@@ -6711,7 +7040,7 @@
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Project_ID; schema/doc version; baseline; source revision; author; reviewer; dates; purpose; risk; requested action</t>
+          <t>Project_ID; export ID; audience/profile version; generation time; source Markdown paths/IDs/revisions/hashes; schema/doc version; baseline; purpose; omitted content and full-source links</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
@@ -6721,7 +7050,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Do not conflate template version, artifact version and product release version.</t>
+          <t>Manifest identifies a derived sharing view. Source changes mark the export stale; never infer approval from generation.</t>
         </is>
       </c>
     </row>
@@ -6743,7 +7072,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Type; status; owner; source location; current baseline; supersedes; applicability rationale</t>
+          <t>Type; status; owner; canonical Markdown path/section; current baseline/revision; supersedes; applicability rationale</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -6753,7 +7082,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Exactly one current authoritative location per artifact version.</t>
+          <t>Resolve each artifact to its canonical Markdown record; link authoritative machine schema/diagram sources separately.</t>
         </is>
       </c>
     </row>
@@ -6925,7 +7254,7 @@
       </c>
       <c r="B12" s="6" t="inlineStr">
         <is>
-          <t>ADR Sections</t>
+          <t>ADR Summaries and Source Links</t>
         </is>
       </c>
       <c r="C12" s="6" t="inlineStr">
@@ -6935,17 +7264,17 @@
       </c>
       <c r="D12" s="6" t="inlineStr">
         <is>
-          <t>Narrative text; supporting source ID; optional option ID</t>
+          <t>Decision summary; rationale/consequence summary; canonical ADR path/section/revision; optional narrative extract</t>
         </is>
       </c>
       <c r="E12" s="6" t="inlineStr">
         <is>
-          <t>Design profile when narrative exceeds summary</t>
+          <t>Design/engineering audience when useful</t>
         </is>
       </c>
       <c r="F12" s="6" t="inlineStr">
         <is>
-          <t>Use multiple readable rows instead of truncation or a huge unreadable cell.</t>
+          <t>Complete ADR reasoning and history stay in Markdown; mark excerpts and link the full record.</t>
         </is>
       </c>
     </row>
@@ -7333,7 +7662,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="39" customHeight="1">
+    <row r="25" ht="54" customHeight="1">
       <c r="A25" s="6" t="inlineStr">
         <is>
           <t>WB21</t>
@@ -7351,7 +7680,7 @@
       </c>
       <c r="D25" s="6" t="inlineStr">
         <is>
-          <t>Artifact version; role; person/identity; review type; decision; timestamp; evidence; applicability</t>
+          <t>Source artifact version; reviewer role/identity; feedback kind; proposed decision; timestamp; evidence; reconciliation status</t>
         </is>
       </c>
       <c r="E25" s="6" t="inlineStr">
@@ -7361,7 +7690,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>Typed names and agent-created agreement cells are not signatures or authorization.</t>
+          <t>Feedback is proposed input. Canonical review/approval evidence changes only after explicit review in the existing process; stale exports cannot update current approvals.</t>
         </is>
       </c>
     </row>
@@ -7383,7 +7712,7 @@
       </c>
       <c r="D26" s="6" t="inlineStr">
         <is>
-          <t>Artifact ID; old/new version; reason; impact; status; author; reviewer; evidence</t>
+          <t>Source change ID; artifact ID; old/new revision; reason; impact; reviewer; evidence; feedback/export reference</t>
         </is>
       </c>
       <c r="E26" s="6" t="inlineStr">
@@ -7393,7 +7722,7 @@
       </c>
       <c r="F26" s="6" t="inlineStr">
         <is>
-          <t>Append history, preserve superseded versions and do not carry approval onto changed content.</t>
+          <t>Derive history from versioned source; archive exports. Do not carry approval onto changed content.</t>
         </is>
       </c>
     </row>
@@ -7836,7 +8165,7 @@
       </c>
       <c r="G12" s="7" t="inlineStr"/>
     </row>
-    <row r="13" ht="39" customHeight="1">
+    <row r="13" ht="84" customHeight="1">
       <c r="A13" s="6" t="inlineStr">
         <is>
           <t>REQ09</t>
@@ -7844,22 +8173,22 @@
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>Excel is the current review format</t>
+          <t>Markdown primary; Excel accompanies each relevant audience</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Deliver a useful XLSX with appropriate selected artifact tabs and reviewer fields.</t>
+          <t>Author/version engineering artifacts in Markdown. Export selected audience tables with source paths/IDs/revisions/hashes, audience/profile, generated date, omissions and full-source links. JSON is a derived rendering snapshot.</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>User instruction; F13</t>
+          <t>User correction; F10; F13</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>EV14</t>
+          <t>EV14; EV28; EV29</t>
         </is>
       </c>
       <c r="F13" s="7" t="inlineStr">
@@ -7869,7 +8198,7 @@
       </c>
       <c r="G13" s="7" t="inlineStr"/>
     </row>
-    <row r="14" ht="39" customHeight="1">
+    <row r="14" ht="69" customHeight="1">
       <c r="A14" s="6" t="inlineStr">
         <is>
           <t>REQ10</t>
@@ -7877,12 +8206,12 @@
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>Preserve workbook edits and provenance</t>
+          <t>Preserve feedback without competing editable masters</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
         <is>
-          <t>Round trips preserve IDs, comments/decisions and formulas; stale regeneration is refused.</t>
+          <t>Archive annotated exports; compare feedback by stable source ID/version, flag stale/conflicting input, and review changes into Markdown before regenerating. No automatic source or approval updates.</t>
         </is>
       </c>
       <c r="D14" s="6" t="inlineStr">
@@ -7892,7 +8221,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>EV15; EV16</t>
+          <t>EV15; EV16; EV29</t>
         </is>
       </c>
       <c r="F14" s="7" t="inlineStr">
@@ -7991,7 +8320,7 @@
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>EV19</t>
+          <t>EV19; EV28</t>
         </is>
       </c>
       <c r="F17" s="7" t="inlineStr">
@@ -8263,7 +8592,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:E31"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="17" customWidth="1" min="1" max="1"/>
@@ -8687,7 +9016,7 @@
         </is>
       </c>
     </row>
-    <row r="18" ht="39" customHeight="1">
+    <row r="18" ht="54" customHeight="1">
       <c r="A18" s="6" t="inlineStr">
         <is>
           <t>EV14</t>
@@ -8695,17 +9024,17 @@
       </c>
       <c r="B18" s="6" t="inlineStr">
         <is>
-          <t>Workbook profile</t>
+          <t>Markdown source and audience workbook</t>
         </is>
       </c>
       <c r="C18" s="6" t="inlineStr">
         <is>
-          <t>Author one meaningful feature or release record.</t>
+          <t>Author one meaningful feature/release record in Markdown, then request an audience export.</t>
         </is>
       </c>
       <c r="D18" s="6" t="inlineStr">
         <is>
-          <t>Excel includes relevant tabs, stable IDs, reviewer fields and navigable tables.</t>
+          <t>Markdown contains the complete canonical record; Excel carries relevant navigable tables, stable source IDs/links, profile/version and freshness metadata.</t>
         </is>
       </c>
       <c r="E18" s="6" t="inlineStr">
@@ -8714,7 +9043,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="39" customHeight="1">
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>EV15</t>
@@ -8722,17 +9051,17 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Human edits</t>
+          <t>Workbook feedback reconciliation</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Reviewer changes comment, priority proposal and decision cells.</t>
+          <t>Reviewer comments and proposes a changed priority/decision in an audience workbook.</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Reconcile by ID; preserve changes; stale snapshot cannot overwrite them.</t>
+          <t>Report proposals by source ID/version; preserve original feedback; apply only reviewed changes to Markdown. Workbook agreement never imports source approval.</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
@@ -8741,7 +9070,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="39" customHeight="1">
+    <row r="20" ht="54" customHeight="1">
       <c r="A20" s="6" t="inlineStr">
         <is>
           <t>EV16</t>
@@ -8759,7 +9088,7 @@
       </c>
       <c r="D20" s="6" t="inlineStr">
         <is>
-          <t>Headers, IDs, links, formulas and review cells preserved or differences reported.</t>
+          <t>Source locators, headers, IDs, links, formulas and review cells preserved or differences reported; original annotated workbook remains archived.</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr">
@@ -8849,7 +9178,7 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="39" customHeight="1">
+    <row r="24" ht="54" customHeight="1">
       <c r="A24" s="6" t="inlineStr">
         <is>
           <t>EV20</t>
@@ -8862,12 +9191,12 @@
       </c>
       <c r="C24" s="6" t="inlineStr">
         <is>
-          <t>Export existing PRD/story IDs to Excel then review.</t>
+          <t>Reference existing PRD/story identities through Markdown and export them to Excel.</t>
         </is>
       </c>
       <c r="D24" s="6" t="inlineStr">
         <is>
-          <t>Reuse original IDs/source metadata and validate without generating a competing PRD.</t>
+          <t>Preserve engine identities/source metadata through the adapter, identify authoritative machine fields and avoid a competing PRD or workbook master.</t>
         </is>
       </c>
       <c r="E24" s="6" t="inlineStr">
@@ -9062,6 +9391,60 @@
       <c r="E31" s="6" t="inlineStr">
         <is>
           <t>REQ20</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="54" customHeight="1">
+      <c r="A32" s="6" t="inlineStr">
+        <is>
+          <t>EV28</t>
+        </is>
+      </c>
+      <c r="B32" s="6" t="inlineStr">
+        <is>
+          <t>Audience projection</t>
+        </is>
+      </c>
+      <c r="C32" s="6" t="inlineStr">
+        <is>
+          <t>Export the same baseline for product, engineering, QA/UAT, operations and executive audiences.</t>
+        </is>
+      </c>
+      <c r="D32" s="6" t="inlineStr">
+        <is>
+          <t>Each profile selects useful fields/views and declares omissions/full-source links; relevant blockers, limitations, uncertainty and trace IDs survive every applicable projection.</t>
+        </is>
+      </c>
+      <c r="E32" s="6" t="inlineStr">
+        <is>
+          <t>REQ09; REQ13</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="54" customHeight="1">
+      <c r="A33" s="6" t="inlineStr">
+        <is>
+          <t>EV29</t>
+        </is>
+      </c>
+      <c r="B33" s="6" t="inlineStr">
+        <is>
+          <t>Stale source or conflicting feedback</t>
+        </is>
+      </c>
+      <c r="C33" s="6" t="inlineStr">
+        <is>
+          <t>Change Markdown after export; return two conflicting annotated exports.</t>
+        </is>
+      </c>
+      <c r="D33" s="6" t="inlineStr">
+        <is>
+          <t>Compare source revisions/hashes, report staleness/conflicts, preserve both inputs and require review against current source before changes. No silent import or overwrite.</t>
+        </is>
+      </c>
+      <c r="E33" s="6" t="inlineStr">
+        <is>
+          <t>REQ09; REQ10</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
feat: add local engineering artifact exports and feedback tooling
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
@@ -769,7 +769,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Research and proposed update only; no catalogue or runtime changes are implemented.</t>
+          <t>Research and update plan; P01 contracts and P02 opt-in local tooling delivered; catalogue skills remain pending.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.2 / Draft for review</t>
+          <t>0.3 / Draft for review</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>User authorized research followed by planning</t>
+          <t>User authorized research, planning and subsequent P01/P02 delivery</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Implementation, installation, remote publishing and deployment are separate stages.</t>
+          <t>Local tooling implemented; installation, remote publishing and deployment remain separate stages.</t>
         </is>
       </c>
     </row>
@@ -1040,7 +1040,7 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="39" customHeight="1">
+    <row r="19" ht="54" customHeight="1">
       <c r="A19" s="6" t="inlineStr">
         <is>
           <t>Next action</t>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>Review delivered P01 content/source and audience export contracts</t>
+          <t>P03 focused authoring and workbook skills</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Then implement P02 bounded exporter/feedback tooling; later focused skills remain outstanding.</t>
+          <t>Reuse delivered P01/P02 contracts, source adapters, usage and regression evidence; discovery, pilots and reviewed integration follow.</t>
         </is>
       </c>
     </row>
@@ -1074,7 +1074,7 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="54" customHeight="1">
+    <row r="21" ht="39" customHeight="1">
       <c r="A21" s="6" t="inlineStr">
         <is>
           <t>Audience</t>
@@ -1087,7 +1087,7 @@
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>Other audience profiles are defined in 14 Audience Profiles for later implementation; this helper renders this review package only.</t>
+          <t>Generic profiles are implemented by the separate P02 tool; this helper renders this review package only.</t>
         </is>
       </c>
     </row>
@@ -1244,7 +1244,7 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>P01 contract/examples delivered locally for review; implementation deferred</t>
+          <t>P01 contract/examples delivered locally; P02 tooling now available</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
@@ -1264,7 +1264,7 @@
       </c>
       <c r="F5" s="6" t="inlineStr">
         <is>
-          <t>Delivered explicit source/identity/content/audience/freshness/feedback contracts, native-engine mapping and tiny/feature/ADR/release examples; detailed design pending review. P02 functional behaviors remain unimplemented.</t>
+          <t>Delivered explicit source/identity/content/audience/freshness/feedback contracts, native-engine mapping and tiny/feature/ADR/release examples; detailed design pending review. P02 functional behaviors now delivered separately; project pilots remain pending.</t>
         </is>
       </c>
       <c r="G5" s="6" t="inlineStr">
@@ -1281,7 +1281,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>Markdown-to-Excel export and feedback reporting</t>
+          <t>Local export and feedback tooling delivered for review</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -1291,7 +1291,7 @@
       </c>
       <c r="D6" s="6" t="inlineStr">
         <is>
-          <t>Proposed karakana/tools/engineering_artifacts.py; tests/test_engineering_artifacts_workbooks.py; chosen optional dependency group in pyproject.toml</t>
+          <t>karakana/tools/engineering_artifacts.py; tests/test_engineering_artifacts.py; optional workbooks dependency in pyproject.toml; P02.md usage and verification</t>
         </is>
       </c>
       <c r="E6" s="6" t="inlineStr">
@@ -1301,7 +1301,7 @@
       </c>
       <c r="F6" s="6" t="inlineStr">
         <is>
-          <t>Functional fixtures prove source/export parity, audience omissions and blocker visibility, traceability, literal text, freshness, conflicting feedback, no-overwrite and office round trips.</t>
+          <t>47 focused tests cover source/export parity, audience omissions/blockers, literal text, freshness, conflicting feedback and no-overwrite. Local CLI and LibreOffice round trip verified; Excel desktop and real project pilots pending.</t>
         </is>
       </c>
       <c r="G6" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat: add experimental engineering documentation skills
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
@@ -761,7 +761,7 @@
         </is>
       </c>
     </row>
-    <row r="2" ht="32" customHeight="1">
+    <row r="2" ht="45" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
           <t>Purpose</t>
@@ -769,7 +769,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Research and update plan; P01 contracts and P02 opt-in local tooling delivered; catalogue skills remain pending.</t>
+          <t>Research and update plan; P01 contracts, P02 local tooling and P03 experimental skills delivered; discovery/pilots/integration pending.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.3 / Draft for review</t>
+          <t>0.4 / Local delivery for review</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -853,7 +853,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="39" customHeight="1">
+    <row r="8" ht="54" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Authority</t>
@@ -861,12 +861,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>User authorized research, planning and subsequent P01/P02 delivery</t>
+          <t>User authorized research, planning and subsequent P01–P03 delivery</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Local tooling implemented; installation, remote publishing and deployment remain separate stages.</t>
+          <t>Local tooling and experimental skills implemented; personal installation, remote publishing and deployment remain separate stages.</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>P03 focused authoring and workbook skills</t>
+          <t>P04 discovery and optional project enablement</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Reuse delivered P01/P02 contracts, source adapters, usage and regression evidence; discovery, pilots and reviewed integration follow.</t>
+          <t>Reuse delivered P01–P03 contracts, tools, experimental skills and verification; generated index/global pointers and narrow skillpack selection, then pilots/integration.</t>
         </is>
       </c>
     </row>
@@ -1318,7 +1318,7 @@
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>Focused authoring skills and original references</t>
+          <t>Five experimental skills and original references delivered locally</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
@@ -1328,7 +1328,7 @@
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Proposed skills/engineering-requirements/; engineering-design-records/; engineering-delivery-planning/; engineering-release-documentation/; engineering-workbooks/</t>
+          <t>skills/engineering-requirements/; engineering-design-records/; engineering-delivery-planning/; engineering-release-documentation/; engineering-workbooks/; tests/test_engineering_documentation_skills.py; P03.md</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
@@ -1338,7 +1338,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>Validate all skills; focused evals; source/license register; no proprietary skill text bundled.</t>
+          <t>Five valid/loadable experimental skills; 14 conditional guides; four neutral examples/23 records; 19 coverage evals and 16 integration tests pass. Full suite 641 tests and 166 evals pass; original source/license register. No stable promotion or model-behavior claim.</t>
         </is>
       </c>
       <c r="G7" s="6" t="inlineStr">
@@ -6674,7 +6674,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Names and boundaries are proposed; no new skills have been created.</t>
+          <t>Five original experimental skills created by P03; independent review and project pilots pending.</t>
         </is>
       </c>
     </row>
@@ -6898,7 +6898,7 @@
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>references/workbook-contract.md; audience-profiles.md; assets/export templates; tool adapter; evals</t>
+          <t>references/workbook-contract.md; audience-profiles.md; shared existing template/P02 tool; evals</t>
         </is>
       </c>
       <c r="F9" s="7" t="inlineStr">

</xml_diff>

<commit_message>
feat: expose engineering documentation skills in catalogue and project profiles
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
@@ -769,7 +769,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Research and update plan; P01 contracts, P02 local tooling and P03 experimental skills delivered; discovery/pilots/integration pending.</t>
+          <t>Research and update plan; P01 contracts, P02 local tooling, P03 experimental skills and P04 discovery delivered; pilots/integration pending.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.4 / Local delivery for review</t>
+          <t>0.5 / Local delivery for review</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>User authorized research, planning and subsequent P01–P03 delivery</t>
+          <t>User authorized research, planning and subsequent P01–P04 delivery</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Local tooling and experimental skills implemented; personal installation, remote publishing and deployment remain separate stages.</t>
+          <t>Local tooling, experimental skills and discovery implemented; personal installation, remote publishing and deployment remain separate stages.</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>P04 discovery and optional project enablement</t>
+          <t>P05 controlled authoring/export/review pilots</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Reuse delivered P01–P03 contracts, tools, experimental skills and verification; generated index/global pointers and narrow skillpack selection, then pilots/integration.</t>
+          <t>Reuse delivered P01–P04 contracts, tools, skills and discovery; select neutral scenarios and evidence/audience verification, then reviewed integration.</t>
         </is>
       </c>
     </row>
@@ -1355,7 +1355,7 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>Global discovery and narrow project enablement</t>
+          <t>Global discovery and narrow project enablement delivered locally</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
@@ -1365,17 +1365,17 @@
       </c>
       <c r="D8" s="6" t="inlineStr">
         <is>
-          <t>skills/README.md generated index; docs/engineering-process.md pointer; ubongo/global/engineering-standards.md; skillpacks/karakana.yml; lims.yml; ent-meal.yml</t>
+          <t>skills/README.md generated index; docs/engineering-process.md pointer; ubongo/global/engineering-standards.md; skillpacks/karakana.yml; lims.yml; ent-meal.yml; tests/test_engineering_skill_discovery.py; P04.md</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr">
         <is>
-          <t>Regenerate index through supported CLI; add concise applicability pointers; select optional skills for relevant packs. Avoid mandatory loading on unrelated tasks; do not alter model routing or existing protocol approval rules.</t>
+          <t>Regenerated index and concise applicability pointers; five optional choices in three packs. Explicit selection loads one skill body and current project memory; defaults, routing and approval rules unchanged.</t>
         </is>
       </c>
       <c r="F8" s="6" t="inlineStr">
         <is>
-          <t>Skill/skillpack/memory validation; representative selection evals; review global/project boundaries.</t>
+          <t>21 selection/index/isolation checks and five instruction/config evals pass; full 662 tests and 171 evals pass. Skills/packs and three project memories valid; source coverage is not agent-behavior evidence.</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr">

</xml_diff>

<commit_message>
docs: deliver controlled engineering artifact and workbook pilots
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
@@ -769,7 +769,7 @@
       </c>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Research and update plan; P01 contracts, P02 local tooling, P03 experimental skills and P04 discovery delivered; pilots/integration pending.</t>
+          <t>Research and update plan; P01 contracts, P02 local tooling, P03 experimental skills, P04 discovery and P05 controlled pilots delivered; reviewed integration pending.</t>
         </is>
       </c>
     </row>
@@ -827,7 +827,7 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.5 / Local delivery for review</t>
+          <t>0.6 / Local delivery for review</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
@@ -861,12 +861,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>User authorized research, planning and subsequent P01–P04 delivery</t>
+          <t>User authorized research, planning and subsequent P01–P05 delivery</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Local tooling, experimental skills and discovery implemented; personal installation, remote publishing and deployment remain separate stages.</t>
+          <t>Local tooling, experimental skills, discovery and controlled pilots implemented; personal installation, remote publishing and deployment remain separate stages.</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>P05 controlled authoring/export/review pilots</t>
+          <t>P06 independent review and authorized integration</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Reuse delivered P01–P04 contracts, tools, skills and discovery; select neutral scenarios and evidence/audience verification, then reviewed integration.</t>
+          <t>Reuse delivered P01–P05 contracts, tools, skills, discovery and pilot QA; inspect full diff, address findings and prepare concrete PR; existing remote-action authority applies.</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="84" customHeight="1">
+    <row r="9" ht="99" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
           <t>P05</t>
@@ -1392,7 +1392,7 @@
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>Prove useful output with controlled pilots</t>
+          <t>Controlled authoring/export/review pilots delivered locally</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
@@ -1402,17 +1402,17 @@
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Synthetic fixtures; skills/*/evals/; workbook QA report; docs/engineering-artifacts.md</t>
+          <t>pilots/ brief, four original Markdown documents, machine fixtures, retained requirement amendment, six XLSX/JSON pairs, QA.md/observations/preview; tests/test_engineering_artifact_pilots.py; P05.md</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>Author complete synthetic requirements/stories, ADR/design and roadmap/release records in Markdown. Export by audience; validate/render Excel; test source freshness and reviewed feedback reconciliation. A LIMS release pack remains a later requested application.</t>
+          <t>Authored complete neutral scenario from resolved seed; five profiles retain blockers/source authority. Explicit reviewed wording amendment preserves IDs/history. Six actual feedback exercises and six office roundtrips; existing profile 0.1 retained as author-assessed review baseline. Real LIMS release pack remains separate.</t>
         </is>
       </c>
       <c r="F9" s="6" t="inlineStr">
         <is>
-          <t>Source-to-export parity, useful audience views, preserved blockers/limitations, actual office/feedback results and accessibility limits recorded; agree profile baseline.</t>
+          <t>14 functional checks; 676 full tests; 171 deterministic evals pass. Seven-source hash/parity and six LibreOffice returns unchanged semantically; readiness PDF visually inspected. Self-review only; native Excel/assistive, audience sign-off, independent review and real application pending.</t>
         </is>
       </c>
       <c r="G9" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Review engineering catalogue and bound workbook feedback scans
</commit_message>
<xml_diff>
--- a/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
+++ b/docs/skills/engineering-artifact-catalogue/research-and-update-plan.xlsx
@@ -827,12 +827,12 @@
       </c>
       <c r="B6" s="6" t="inlineStr">
         <is>
-          <t>0.6 / Local delivery for review</t>
+          <t>0.7 / Catalogue review for integration</t>
         </is>
       </c>
       <c r="C6" s="6" t="inlineStr">
         <is>
-          <t>Research conclusions and implementation proposal; no approval implied.</t>
+          <t>Research, local delivery and author review; no independent approval or stable promotion implied.</t>
         </is>
       </c>
     </row>
@@ -853,7 +853,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="54" customHeight="1">
+    <row r="8" ht="69" customHeight="1">
       <c r="A8" s="6" t="inlineStr">
         <is>
           <t>Authority</t>
@@ -861,12 +861,12 @@
       </c>
       <c r="B8" s="6" t="inlineStr">
         <is>
-          <t>User authorized research, planning and subsequent P01–P05 delivery</t>
+          <t>User authorized research, planning, P01–P05 delivery and P06 review/PR integration</t>
         </is>
       </c>
       <c r="C8" s="6" t="inlineStr">
         <is>
-          <t>Local tooling, experimental skills, discovery and controlled pilots implemented; personal installation, remote publishing and deployment remain separate stages.</t>
+          <t>Local delivery and author review completed; publish the reviewed task branch/PR, then verify actual CI and human-review gates. Personal installation, deployment and real release drafting remain separate.</t>
         </is>
       </c>
     </row>
@@ -1048,12 +1048,12 @@
       </c>
       <c r="B19" s="6" t="inlineStr">
         <is>
-          <t>P06 independent review and authorized integration</t>
+          <t>Review the concrete P06 PR and squash when its gates are satisfied</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Reuse delivered P01–P05 contracts, tools, skills, discovery and pilot QA; inspect full diff, address findings and prepare concrete PR; existing remote-action authority applies.</t>
+          <t>Reuse P06.md for resolved findings, exact verification and limitations. Check actual head/base, CI and human review; do not infer independent approval from continuing author review.</t>
         </is>
       </c>
     </row>
@@ -1421,7 +1421,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="69" customHeight="1">
+    <row r="10" ht="99" customHeight="1">
       <c r="A10" s="6" t="inlineStr">
         <is>
           <t>P06</t>
@@ -1429,7 +1429,7 @@
       </c>
       <c r="B10" s="6" t="inlineStr">
         <is>
-          <t>Review and integrate accepted catalogue change</t>
+          <t>Catalogue author review and PR preparation; remote gates pending</t>
         </is>
       </c>
       <c r="C10" s="6" t="inlineStr">
@@ -1439,22 +1439,22 @@
       </c>
       <c r="D10" s="6" t="inlineStr">
         <is>
-          <t>Final diff, generated index, test/eval/validation reports, task trace and handoff</t>
+          <t>P06.md; complete upstream diff; five regression cases; generated research pack 0.7; isolated gates; task traces and append-only handoff</t>
         </is>
       </c>
       <c r="E10" s="6" t="inlineStr">
         <is>
-          <t>Use skill-update protocol for metadata/guidance work and python-code-change for deterministic tools; run required suite in isolated runtime; review safety/provenance; publish PR and squash only when authorized.</t>
+          <t>Resolved sparse workbook scan and dropped blank-row comments; shared 500,000-cell import/export limit; original input bytes preserved. Five skills remain experimental/optional; blank templates remain generic. Publish reviewed task branch/PR, inspect actual CI/review and squash only with required authority.</t>
         </is>
       </c>
       <c r="F10" s="6" t="inlineStr">
         <is>
-          <t>No P0/P1 unresolved; CI and human review as required; state local/merged/installed separately; promotion remains evidence-based.</t>
+          <t>New five regressions and all 52 focused tool tests pass. Full gate results are recorded in P06.md. No unresolved author-review P0/P1; CI, human review, real project/native Excel usability and stable promotion remain separate evidence.</t>
         </is>
       </c>
       <c r="G10" s="6" t="inlineStr">
         <is>
-          <t>REQ01; REQ12; REQ19</t>
+          <t>REQ01; REQ10; REQ11; REQ12; REQ18; REQ19</t>
         </is>
       </c>
     </row>

</xml_diff>